<commit_message>
Fixed small issue in frametime graph
</commit_message>
<xml_diff>
--- a/Experiment/Results/ComparingData.xlsx
+++ b/Experiment/Results/ComparingData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Howest\GD_J3_S2\Gradwork_2.0\Gradwork\Experiment\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2991C71-C374-4CA1-98AB-3C4CCC8A899F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB151099-D761-4768-836B-C788229CF40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Frametime" sheetId="1" r:id="rId1"/>
@@ -624,7 +624,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -1595,7 +1594,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-GB"/>
-              <a:t>3840/2054</a:t>
+              <a:t>3840*2054</a:t>
             </a:r>
           </a:p>
         </c:rich>

</xml_diff>

<commit_message>
Added "comparing data" section
</commit_message>
<xml_diff>
--- a/Experiment/Results/ComparingData.xlsx
+++ b/Experiment/Results/ComparingData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Howest\GD_J3_S2\Gradwork_2.0\Gradwork\Experiment\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB151099-D761-4768-836B-C788229CF40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138ADF52-4C69-4366-B51E-E35077559EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22590" yWindow="-10680" windowWidth="16430" windowHeight="12340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Frametime" sheetId="1" r:id="rId1"/>
@@ -394,7 +394,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.12548381452318461"/>
+          <c:y val="0.16245370370370371"/>
+          <c:w val="0.84396062992125986"/>
+          <c:h val="0.51681284631087776"/>
+        </c:manualLayout>
+      </c:layout>
       <c:lineChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
@@ -624,6 +634,7 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -4775,6 +4786,17 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SSAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -4787,6 +4809,27 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>VRAM!$C$8:$F$8</c:f>
@@ -4818,6 +4861,17 @@
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>HBAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -4830,6 +4884,27 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>VRAM!$C$9:$F$9</c:f>
@@ -4861,6 +4936,17 @@
         <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>GTAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -4873,6 +4959,27 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>VRAM!$C$10:$F$10</c:f>
@@ -5302,6 +5409,17 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SSAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -5314,6 +5432,27 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>VRAM!$C$13:$F$13</c:f>
@@ -5345,6 +5484,17 @@
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>HBAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -5357,6 +5507,27 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>VRAM!$C$14:$F$14</c:f>
@@ -5388,6 +5559,17 @@
         <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>GTAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -5400,6 +5582,27 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>VRAM!$C$15:$F$15</c:f>

</xml_diff>

<commit_message>
Added discussion section to paper
</commit_message>
<xml_diff>
--- a/Experiment/Results/ComparingData.xlsx
+++ b/Experiment/Results/ComparingData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Howest\GD_J3_S2\Gradwork_2.0\Gradwork\Experiment\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138ADF52-4C69-4366-B51E-E35077559EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79627AAF-DD50-4125-81DA-A16175B76453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22590" yWindow="-10680" windowWidth="16430" windowHeight="12340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Frametime" sheetId="1" r:id="rId1"/>
@@ -634,7 +634,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -860,6 +859,1875 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="424388192"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>800*600</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14978572829429709"/>
+          <c:y val="0.17171296296296296"/>
+          <c:w val="0.82106747785302669"/>
+          <c:h val="0.60623549024875822"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SSAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$2:$F$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$3:$F$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>261</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E758-4968-B983-99CC030AAE97}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>HBAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$2:$F$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$4:$F$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>261</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E758-4968-B983-99CC030AAE97}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>GTAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$2:$F$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$5:$F$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>261</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>261</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-E758-4968-B983-99CC030AAE97}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1275306000"/>
+        <c:axId val="1275308080"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1275306000"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Samples</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.43264315728419478"/>
+              <c:y val="0.85318163969661276"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1275308080"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1275308080"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Usage in mb</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1275306000"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>1920*991</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14978572829429709"/>
+          <c:y val="0.17171296296296296"/>
+          <c:w val="0.82106747785302669"/>
+          <c:h val="0.60623549024875822"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SSAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$8:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>477</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>477</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>477</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>477</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4327-4DC4-BBB2-35F6AFD3AF67}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>HBAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$9:$F$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>476</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>476</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>476</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>476</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-4327-4DC4-BBB2-35F6AFD3AF67}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>GTAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$10:$F$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>476</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>476</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>476</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>476</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-4327-4DC4-BBB2-35F6AFD3AF67}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1275306000"/>
+        <c:axId val="1275308080"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1275306000"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Samples</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.43264315728419478"/>
+              <c:y val="0.85318163969661276"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1275308080"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1275308080"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Usage in mb</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1275306000"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>3840*2054</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14978572829429709"/>
+          <c:y val="0.17171296296296296"/>
+          <c:w val="0.82106747785302669"/>
+          <c:h val="0.60623549024875822"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SSAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$13:$F$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1331</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1331</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1331</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1331</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DDA8-40E5-A8F4-5EA81805BD61}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>HBAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$14:$F$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1330</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1330</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1330</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1330</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-DDA8-40E5-A8F4-5EA81805BD61}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>VRAM!$B$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>GTAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>VRAM!$C$15:$F$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1330</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1330</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1330</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1330</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-DDA8-40E5-A8F4-5EA81805BD61}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1275306000"/>
+        <c:axId val="1275308080"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1275306000"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Samples</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.43264315728419478"/>
+              <c:y val="0.85318163969661276"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1275308080"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1275308080"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Usage in mb</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1275306000"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3538,11 +5406,11 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="1"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>CPU!$B$3</c:f>
+              <c:f>CPU!$B$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3554,7 +5422,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent1"/>
+                <a:srgbClr val="00B0F0"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3565,7 +5433,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>CPU!$C$2:$F$2</c:f>
+              <c:f>CPU!$C$12:$F$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3586,96 +5454,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>CPU!$C$3:$F$3</c:f>
+              <c:f>CPU!$C$13:$F$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>514.9</c:v>
+                  <c:v>1290</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>514.70000000000005</c:v>
+                  <c:v>1306.0999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>528.29999999999995</c:v>
+                  <c:v>1303</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>524</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2B46-4AEB-89F5-CD01F8AA34E8}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>CPU!$B$4</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>HBAO</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:numRef>
-              <c:f>CPU!$C$2:$F$2</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>CPU!$C$4:$F$4</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>514.20000000000005</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>514.29999999999995</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>524.6</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>514.70000000000005</c:v>
+                  <c:v>1299.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3689,14 +5482,14 @@
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>CPU!$B$5</c:f>
+              <c:f>CPU!$B$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>GTAO</c:v>
+                  <c:v>HBAO</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3704,7 +5497,10 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent3"/>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3715,7 +5511,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>CPU!$C$2:$F$2</c:f>
+              <c:f>CPU!$C$12:$F$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3736,21 +5532,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>CPU!$C$5:$F$5</c:f>
+              <c:f>CPU!$C$14:$F$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>515.6</c:v>
+                  <c:v>1304.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>515.6</c:v>
+                  <c:v>1299</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>518.29999999999995</c:v>
+                  <c:v>1297.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>523.5</c:v>
+                  <c:v>1287.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3759,6 +5555,83 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-2B46-4AEB-89F5-CD01F8AA34E8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>CPU!$B$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>GTAO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>CPU!$C$12:$F$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3600</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>CPU!$C$15:$F$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1287.9000000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1295.9000000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1290.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1299.5999999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-383F-4BEE-8C0B-B23FC2048952}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4161,11 +6034,11 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="1"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$3</c:f>
+              <c:f>CPU!$B$3</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4188,42 +6061,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$2:$F$2</c:f>
+              <c:f>CPU!$C$2:$D$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$3:$F$3</c:f>
+              <c:f>CPU!$C$3:$D$3</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>261</c:v>
+                  <c:v>514.9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>261</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>261</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>261</c:v>
+                  <c:v>514.70000000000005</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4231,16 +6092,16 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E758-4968-B983-99CC030AAE97}"/>
+              <c16:uniqueId val="{00000001-A164-4DF4-A241-52C17B28A3EA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="1"/>
+          <c:idx val="2"/>
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$4</c:f>
+              <c:f>CPU!$B$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4263,42 +6124,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$2:$F$2</c:f>
+              <c:f>CPU!$C$2:$D$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$4:$F$4</c:f>
+              <c:f>CPU!$C$4:$D$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>261</c:v>
+                  <c:v>514.20000000000005</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>261</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>261</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>261</c:v>
+                  <c:v>514.29999999999995</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4306,16 +6155,16 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E758-4968-B983-99CC030AAE97}"/>
+              <c16:uniqueId val="{00000002-A164-4DF4-A241-52C17B28A3EA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="2"/>
+          <c:idx val="3"/>
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$5</c:f>
+              <c:f>CPU!$B$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4338,42 +6187,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$2:$F$2</c:f>
+              <c:f>CPU!$C$2:$D$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$5:$F$5</c:f>
+              <c:f>CPU!$C$5:$D$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>261</c:v>
+                  <c:v>515.6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>261</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>261</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>261</c:v>
+                  <c:v>515.6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4381,7 +6218,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-E758-4968-B983-99CC030AAE97}"/>
+              <c16:uniqueId val="{00000004-A164-4DF4-A241-52C17B28A3EA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4784,11 +6621,11 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="1"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$13</c:f>
+              <c:f>CPU!$B$8</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4811,42 +6648,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:f>CPU!$C$7:$D$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$8:$F$8</c:f>
+              <c:f>CPU!$C$8:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>477</c:v>
+                  <c:v>687.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>477</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>477</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>477</c:v>
+                  <c:v>702.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4854,16 +6679,16 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4327-4DC4-BBB2-35F6AFD3AF67}"/>
+              <c16:uniqueId val="{00000001-8B73-4482-AEEE-7686D3A89B7B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="1"/>
+          <c:idx val="2"/>
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$14</c:f>
+              <c:f>CPU!$B$9</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4886,42 +6711,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:f>CPU!$C$7:$D$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$9:$F$9</c:f>
+              <c:f>CPU!$C$9:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>476</c:v>
+                  <c:v>686.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>476</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>476</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>476</c:v>
+                  <c:v>692</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4929,16 +6742,16 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4327-4DC4-BBB2-35F6AFD3AF67}"/>
+              <c16:uniqueId val="{00000002-8B73-4482-AEEE-7686D3A89B7B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="2"/>
+          <c:idx val="3"/>
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$15</c:f>
+              <c:f>CPU!$B$10</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4961,42 +6774,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$7:$F$7</c:f>
+              <c:f>CPU!$C$7:$D$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$10:$F$10</c:f>
+              <c:f>CPU!$C$10:$D$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>476</c:v>
+                  <c:v>686.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>476</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>476</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>476</c:v>
+                  <c:v>690.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5004,7 +6805,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-4327-4DC4-BBB2-35F6AFD3AF67}"/>
+              <c16:uniqueId val="{00000004-8B73-4482-AEEE-7686D3A89B7B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5407,11 +7208,11 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="2"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$13</c:f>
+              <c:f>CPU!$B$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5423,7 +7224,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent1"/>
+                <a:srgbClr val="00B0F0"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -5434,42 +7235,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:f>CPU!$C$12:$D$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$13:$F$13</c:f>
+              <c:f>CPU!$C$13:$D$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1331</c:v>
+                  <c:v>1290</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1331</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1331</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1331</c:v>
+                  <c:v>1306.0999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5477,16 +7266,16 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-DDA8-40E5-A8F4-5EA81805BD61}"/>
+              <c16:uniqueId val="{00000001-9E0B-49AA-ACBD-284AC5B6918D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="1"/>
+          <c:idx val="3"/>
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$14</c:f>
+              <c:f>CPU!$B$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5498,7 +7287,10 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent2"/>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -5509,42 +7301,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:f>CPU!$C$12:$D$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$14:$F$14</c:f>
+              <c:f>CPU!$C$14:$D$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1330</c:v>
+                  <c:v>1304.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1330</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1330</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1330</c:v>
+                  <c:v>1299</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5552,16 +7332,16 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-DDA8-40E5-A8F4-5EA81805BD61}"/>
+              <c16:uniqueId val="{00000002-9E0B-49AA-ACBD-284AC5B6918D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="2"/>
+          <c:idx val="0"/>
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>VRAM!$B$15</c:f>
+              <c:f>CPU!$B$15</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5573,7 +7353,9 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent3"/>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -5584,42 +7366,30 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>VRAM!$C$12:$F$12</c:f>
+              <c:f>CPU!$C$12:$D$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>VRAM!$C$15:$F$15</c:f>
+              <c:f>CPU!$C$15:$D$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1330</c:v>
+                  <c:v>1287.9000000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1330</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1330</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1330</c:v>
+                  <c:v>1295.9000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5627,7 +7397,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-DDA8-40E5-A8F4-5EA81805BD61}"/>
+              <c16:uniqueId val="{00000004-9E0B-49AA-ACBD-284AC5B6918D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5945,6 +7715,126 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors11.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors12.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -6820,6 +8710,1554 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style11.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style12.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
@@ -11172,6 +14610,120 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>273050</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>74930</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>189230</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A4A2180-0F48-4D95-9893-284E963B2510}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>280670</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>13970</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>196850</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>173990</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE05173D-8937-474D-97D8-7FF56D3B4669}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D0AF30B-E49B-406A-9667-9316A615898B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>